<commit_message>
Actualizacion automatica de mejoras y correcciones
</commit_message>
<xml_diff>
--- a/Plantilla_SaaS_LinPro.xlsx
+++ b/Plantilla_SaaS_LinPro.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lindley-Adm\OneDrive\Desktop\PROYECTOS LIN\LIN_PRO_X_WEB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACC033D6-3D01-4675-84FD-D4C193DB6A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A40CCFAF-342B-451F-ADA9-BBBF15AFCD90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="2" xr2:uid="{A40B6391-4749-4BF0-871F-ADE56F8B4F09}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A40B6391-4749-4BF0-871F-ADE56F8B4F09}"/>
   </bookViews>
   <sheets>
     <sheet name="Insumos" sheetId="1" r:id="rId1"/>
@@ -44,8 +44,67 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Lindley-Adm</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{EF25B4E8-D414-43E2-A2D2-7EDE0536CCF7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Lindley-Adm:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Formula por % colocar la presentacion en: LOTE/GRANEL = 100</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{D674A1CB-DF49-4AC3-B0C3-8F41C91C5B9E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Lindley-Adm:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Formula por % colocar el precio = $0
+(o el precio por litro/kilo)</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="60">
   <si>
     <t>Nombre</t>
   </si>
@@ -68,30 +127,9 @@
     <t>Precio</t>
   </si>
   <si>
-    <t>Shampoo de Coco</t>
-  </si>
-  <si>
-    <t>250ml</t>
-  </si>
-  <si>
-    <t>Extracto de Coco</t>
-  </si>
-  <si>
     <t>Materia Prima</t>
   </si>
   <si>
-    <t>ml</t>
-  </si>
-  <si>
-    <t>Envase 250ml</t>
-  </si>
-  <si>
-    <t>Envases y Empaques</t>
-  </si>
-  <si>
-    <t>und</t>
-  </si>
-  <si>
     <t>Producto_Base</t>
   </si>
   <si>
@@ -102,6 +140,150 @@
   </si>
   <si>
     <t>Cantidad</t>
+  </si>
+  <si>
+    <t>ACIDO OLEICO</t>
+  </si>
+  <si>
+    <t>gr</t>
+  </si>
+  <si>
+    <t>NONIL FENOL 10M</t>
+  </si>
+  <si>
+    <t>FRAGANCIA LAVADORA</t>
+  </si>
+  <si>
+    <t>EDTA</t>
+  </si>
+  <si>
+    <t>COLORANTE AZUL VEGETAL</t>
+  </si>
+  <si>
+    <t>AGUA DESTILADA</t>
+  </si>
+  <si>
+    <t>COMPLEMENTO OPTICO</t>
+  </si>
+  <si>
+    <t>DIETANOLAMINA DE COCO</t>
+  </si>
+  <si>
+    <t>EXTRACTO DE SABILA</t>
+  </si>
+  <si>
+    <t>POLICUAR H-80</t>
+  </si>
+  <si>
+    <t>TENSOACTIVO ANIONICO</t>
+  </si>
+  <si>
+    <t>EXTRACTO DE COCO</t>
+  </si>
+  <si>
+    <t>DEHYQUART-E</t>
+  </si>
+  <si>
+    <t>GENAMIN ACONDICIONANTE</t>
+  </si>
+  <si>
+    <t>PRO-VITAMINA B-5</t>
+  </si>
+  <si>
+    <t>VITAMINA E</t>
+  </si>
+  <si>
+    <t>PLANTAREN</t>
+  </si>
+  <si>
+    <t>EUPERLAND NACARADO</t>
+  </si>
+  <si>
+    <t>TEGOBETINE 1-7</t>
+  </si>
+  <si>
+    <t>METIL PARABENO</t>
+  </si>
+  <si>
+    <t>PROPIL PARABENO</t>
+  </si>
+  <si>
+    <t>ACIDO CITRICO</t>
+  </si>
+  <si>
+    <t>CARBOXIMETILCELULOSA CMC</t>
+  </si>
+  <si>
+    <t>MEDIAMIDE C-90</t>
+  </si>
+  <si>
+    <t>GENAPOL</t>
+  </si>
+  <si>
+    <t>GENAMID</t>
+  </si>
+  <si>
+    <t>COCOAMIDOPROPIL BETAINA</t>
+  </si>
+  <si>
+    <t>TEXAPON NACARADO</t>
+  </si>
+  <si>
+    <t>METIL PARABENO SODICO</t>
+  </si>
+  <si>
+    <t>CLORURO DE SODIO</t>
+  </si>
+  <si>
+    <t>FRAGANCIA SHAMPOO FRUTAL</t>
+  </si>
+  <si>
+    <t>SHAMPOO PARA LAVADORA</t>
+  </si>
+  <si>
+    <t>Lote/Granel</t>
+  </si>
+  <si>
+    <t>DETERGENTE LIQUIDO TIPO MAS COLOR</t>
+  </si>
+  <si>
+    <t>SHAMPOO NATURAL DE SAVILA</t>
+  </si>
+  <si>
+    <t>SHAMPOO DE COCO NATURAL</t>
+  </si>
+  <si>
+    <t>SHAMPOO SUPER SUAVE PARA BEBES</t>
+  </si>
+  <si>
+    <t>SHAMPOO PROFESIONAL CON VITAMINA E</t>
+  </si>
+  <si>
+    <t>0.01</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>63.89</t>
+  </si>
+  <si>
+    <t>0.4</t>
+  </si>
+  <si>
+    <t>96.1</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>0.15</t>
+  </si>
+  <si>
+    <t>0.13</t>
+  </si>
+  <si>
+    <t>1.5</t>
   </si>
 </sst>
 </file>
@@ -111,7 +293,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;$&quot;\ * #,##0.00_-;\-&quot;$&quot;\ * #,##0.00_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -137,6 +319,19 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -146,7 +341,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -265,12 +460,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
@@ -329,9 +553,6 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -342,6 +563,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -943,8 +1173,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2DE8526C-F54A-49DE-85ED-119800CD78F6}" name="TablaInsumos" displayName="TablaInsumos" ref="A1:E3" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="14" tableBorderDxfId="15" totalsRowBorderDxfId="13" headerRowCellStyle="Moneda">
-  <autoFilter ref="A1:E3" xr:uid="{2DE8526C-F54A-49DE-85ED-119800CD78F6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2DE8526C-F54A-49DE-85ED-119800CD78F6}" name="TablaInsumos" displayName="TablaInsumos" ref="A1:E32" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="14" tableBorderDxfId="15" totalsRowBorderDxfId="13" headerRowCellStyle="Moneda">
+  <autoFilter ref="A1:E32" xr:uid="{2DE8526C-F54A-49DE-85ED-119800CD78F6}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{D87A3C9F-8125-475B-B104-0D45894B8F6C}" name="Nombre" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{1FF1ADE1-C3C2-4B95-92E1-C87B6E4D6E99}" name="Categoria" dataDxfId="11"/>
@@ -957,8 +1187,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9D47CEDF-6E1F-40DD-8B41-ECEA0CDFDF2F}" name="TablaProductos" displayName="TablaProductos" ref="A1:C2" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
-  <autoFilter ref="A1:C2" xr:uid="{9D47CEDF-6E1F-40DD-8B41-ECEA0CDFDF2F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{9D47CEDF-6E1F-40DD-8B41-ECEA0CDFDF2F}" name="TablaProductos" displayName="TablaProductos" ref="A1:C7" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="5" tableBorderDxfId="6" totalsRowBorderDxfId="4">
+  <autoFilter ref="A1:C7" xr:uid="{9D47CEDF-6E1F-40DD-8B41-ECEA0CDFDF2F}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{4BF5BD62-7375-46ED-9177-52A52407C7D9}" name="Nombre" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{773DF755-906A-4599-A7F6-4039A025C913}" name="Presentacion" dataDxfId="2"/>
@@ -969,8 +1199,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC2F55FF-9B0A-402D-A54F-6331A6B5F69D}" name="TablaFormulas" displayName="TablaFormulas" ref="A1:D3" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="22" tableBorderDxfId="23" totalsRowBorderDxfId="21">
-  <autoFilter ref="A1:D3" xr:uid="{FC2F55FF-9B0A-402D-A54F-6331A6B5F69D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FC2F55FF-9B0A-402D-A54F-6331A6B5F69D}" name="TablaFormulas" displayName="TablaFormulas" ref="A1:D39" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="22" tableBorderDxfId="23" totalsRowBorderDxfId="21">
+  <autoFilter ref="A1:D39" xr:uid="{FC2F55FF-9B0A-402D-A54F-6331A6B5F69D}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{40C8B78B-D7E0-4BA5-B934-C821B6C62578}" name="Producto_Base" dataDxfId="20"/>
     <tableColumn id="2" xr3:uid="{D1D4FDA2-54D6-422E-BB23-B27C06AF1636}" name="Volumen_Lote" dataDxfId="19"/>
@@ -1298,13 +1528,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F2595BA-36AF-4B70-AEAA-A409F43C11E0}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.3984375" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="11.19921875" style="3"/>
-    <col min="4" max="5" width="11.19921875" style="4"/>
+    <col min="4" max="4" width="11.19921875" style="4"/>
+    <col min="5" max="5" width="11.5" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="3" customFormat="1" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
@@ -1326,39 +1557,540 @@
     </row>
     <row r="2" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D2" s="6">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="E2" s="16">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="21">
-        <v>800</v>
-      </c>
-      <c r="E3" s="22">
-        <v>150</v>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="20">
+        <v>1000</v>
+      </c>
+      <c r="E3" s="21">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E4" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E5" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E6" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="6">
+        <v>100</v>
+      </c>
+      <c r="E7" s="16">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E8" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E9" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E11" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E12" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E13" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E14" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E15" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E16" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E17" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E18" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E19" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E20" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E21" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E22" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E23" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E24" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E25" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D26" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E26" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E27" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D28" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E28" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D29" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E29" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E30" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E31" s="16">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" s="6">
+        <v>1000</v>
+      </c>
+      <c r="E32" s="16">
+        <v>10000</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B32" xr:uid="{4DC0CD48-5DC5-4424-81AB-AC9DF8C732CB}">
+      <formula1>"Materia Prima, Envases y Empaques"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C32" xr:uid="{7D3C8FEA-8EE8-4310-B158-6B575689D353}">
+      <formula1>"und, ml, gr, Kg, Oz"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1367,11 +2099,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{498DDBAC-CEB7-4A8B-B45B-818020CB94E3}">
-  <dimension ref="A1:C2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{498DDBAC-CEB7-4A8B-B45B-818020CB94E3}">
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.19921875" customWidth="1"/>
+    <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.3984375" style="3" customWidth="1"/>
     <col min="3" max="3" width="12" style="4" customWidth="1"/>
   </cols>
@@ -1383,35 +2115,91 @@
       <c r="B1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="22" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="12" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="24">
-        <v>25000</v>
+        <v>45</v>
+      </c>
+      <c r="C2" s="23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="26">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0306CBE1-ABBE-4173-92A9-5191CDB92895}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27" customWidth="1"/>
+    <col min="1" max="1" width="35" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.19921875" style="3" customWidth="1"/>
     <col min="3" max="3" width="24.69921875" customWidth="1"/>
     <col min="4" max="4" width="14.59765625" style="3" customWidth="1"/>
@@ -1419,52 +2207,556 @@
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="B2" s="2">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D2" s="8">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="13">
+        <v>100</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="15">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2">
+        <v>100</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="2">
+        <v>100</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="2">
+        <v>100</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="2">
+        <v>100</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="2">
+        <v>100</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="2">
+        <v>100</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B10" s="2">
+        <v>100</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="2">
+        <v>100</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="2">
+        <v>100</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="8">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="8">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="13">
-        <v>1000</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="15">
-        <v>4</v>
+    <row r="16" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="8">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="8">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="8">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="14.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" s="2">
+        <v>12000</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="8">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D24" s="8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B26" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" s="2">
+        <v>4000</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D29" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="8">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D31" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D32" s="8">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B33" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="8">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D36" s="8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D37" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D38" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" s="2">
+        <v>1000</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="8">
+        <v>583</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A3" xr:uid="{84EC5BB3-0A6C-464E-8FBA-3DD8F6591655}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A39" xr:uid="{84EC5BB3-0A6C-464E-8FBA-3DD8F6591655}">
       <formula1>ListaDeProductos</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C3" xr:uid="{65EC7420-171A-4BDB-80B0-5DE3125EB019}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C39" xr:uid="{65EC7420-171A-4BDB-80B0-5DE3125EB019}">
       <formula1>ListaDeInsumos</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>